<commit_message>
pass import siswa jadi otomatis
</commit_message>
<xml_diff>
--- a/admin/template/template.xlsx
+++ b/admin/template/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp2\htdocs\student\admin\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\student\admin\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E6498BB-F062-4199-9CC8-AD460CAA80C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D032EEFE-7F65-4F6B-A8F3-A6A7B93D8C1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{D40B6584-942C-4C15-8925-48533773B1E9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D40B6584-942C-4C15-8925-48533773B1E9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>NIS</t>
   </si>
@@ -52,9 +52,6 @@
   </si>
   <si>
     <t>DATA SISWA SMK MADYA DEPOK</t>
-  </si>
-  <si>
-    <t>PASSWORD</t>
   </si>
 </sst>
 </file>
@@ -145,12 +142,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -178,9 +172,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -218,7 +212,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -324,7 +318,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -466,7 +460,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -486,50 +480,46 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>6</v>
-      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="2"/>
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
@@ -537,7 +527,6 @@
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
@@ -545,7 +534,6 @@
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="1"/>
@@ -553,7 +541,6 @@
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
@@ -561,7 +548,6 @@
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
@@ -569,7 +555,6 @@
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
@@ -577,7 +562,6 @@
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
@@ -585,7 +569,6 @@
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
@@ -593,7 +576,6 @@
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
@@ -601,81 +583,71 @@
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="6">
     <mergeCell ref="A3:F4"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="D6:D7"/>
     <mergeCell ref="E6:E7"/>
-    <mergeCell ref="F6:F7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>